<commit_message>
Impact Damagers + owner force apply for damageable
</commit_message>
<xml_diff>
--- a/Bug Table.xlsx
+++ b/Bug Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UNI-GAMR3540\GAMR3540_P2724211\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D6D8B9-894B-4F04-872C-900A1EF8BA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE1610B-5826-4353-9D47-3C2FA72B0FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5912ADCA-CC98-4984-9306-2733C0A9C225}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Bug Title</t>
   </si>
@@ -85,6 +85,94 @@
   </si>
   <si>
     <t>Explosion code was always running at start.</t>
+  </si>
+  <si>
+    <t>Constant Health Regen Loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After taking damage, health would regenerate as expected. When reaching max health, health would regenerate to max and then would subtract the same damage healed in the next tick. </t>
+  </si>
+  <si>
+    <t>Only run damage code when delta health &lt; 0</t>
+  </si>
+  <si>
+    <t>Player damageable when dead</t>
+  </si>
+  <si>
+    <t>Players could still be hit after dying, meaning the death particles would play again and more death trophies would spawn</t>
+  </si>
+  <si>
+    <t>Projectiles all moved to first hit point</t>
+  </si>
+  <si>
+    <t>When firing multiple projectiles, they would all move to the point that the first projectile hit.</t>
+  </si>
+  <si>
+    <t>I lost my notes on this one. I think it wasn’t setting something correctly.</t>
+  </si>
+  <si>
+    <t>Projectiles phase through objects</t>
+  </si>
+  <si>
+    <t>Projectiles would move through objects that are in their direct path.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolved </t>
+  </si>
+  <si>
+    <t>Projectiles hit owner</t>
+  </si>
+  <si>
+    <t>Projectiles would get stuck on the owner of the projectile, causing self damage.</t>
+  </si>
+  <si>
+    <t>Implemented ignored colliders and multiple raycast hits in new projectile simulation</t>
+  </si>
+  <si>
+    <t>Implemented active projectile array that is linked directly to raycast command index instead of all projectile array.</t>
+  </si>
+  <si>
+    <t>Projectiles were ticking multiple times due to not being correctly terminated. Resolved when projectile hashing and single array was implemented</t>
+  </si>
+  <si>
+    <t>Defibrilator no ammo consumed</t>
+  </si>
+  <si>
+    <t>Defibrilator would not consume ammo when used.</t>
+  </si>
+  <si>
+    <t>Attempting to "fire" the defibrilator will always consume ammo regardless of whether it hits or not.</t>
+  </si>
+  <si>
+    <t>Defibrilator enemy revives</t>
+  </si>
+  <si>
+    <t>Defibrilator can revive enemies when hitting their trophies instead.</t>
+  </si>
+  <si>
+    <t>Defibrilator checks trophy at point of trying to revive rather than relying on cached isFriendly value.</t>
+  </si>
+  <si>
+    <t>Carriable Rotation Zero</t>
+  </si>
+  <si>
+    <t>When carriable rotation has not been assigned/modified, carriables do not rotate at all.</t>
+  </si>
+  <si>
+    <t>Initialised Grab Rotation Offset with Quaternion.Identity</t>
+  </si>
+  <si>
+    <t>Interactable Event Always Triggers</t>
+  </si>
+  <si>
+    <t>Interactables always invoke their events, even when the user releases the interaction key early.</t>
+  </si>
+  <si>
+    <t>Only invokes interactable events when the interaction is completed</t>
+  </si>
+  <si>
+    <t>Note: Only contains the most notable or most recent bugs. I forgot to make note of a lot of smaller ones that arose in the middle of developing features.
+The table provides the title or name of a bug, what happened, whether it was resolved and if there was a resolution for this bug.</t>
   </si>
 </sst>
 </file>
@@ -126,10 +214,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -165,13 +256,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6B7C473A-8E9F-4EBA-B984-899D7ADF84EC}" name="Table1" displayName="Table1" ref="B2:E30" totalsRowShown="0" dataDxfId="0">
-  <autoFilter ref="B2:E30" xr:uid="{6B7C473A-8E9F-4EBA-B984-899D7ADF84EC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6B7C473A-8E9F-4EBA-B984-899D7ADF84EC}" name="Table1" displayName="Table1" ref="B3:E31" totalsRowShown="0" dataDxfId="4">
+  <autoFilter ref="B3:E31" xr:uid="{6B7C473A-8E9F-4EBA-B984-899D7ADF84EC}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B83D2B8A-F268-4DF4-A5BE-50C482361CDE}" name="Bug Title" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{BD499A1D-A0BC-45A1-8345-02C6BCC518BA}" name="Bug Description" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{916FF057-7F24-472E-9D49-1448562FD20E}" name="Resolved?" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{7DCAFC68-52C1-419F-AE79-351C1976AE51}" name="Resolution" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{B83D2B8A-F268-4DF4-A5BE-50C482361CDE}" name="Bug Title" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{BD499A1D-A0BC-45A1-8345-02C6BCC518BA}" name="Bug Description" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{916FF057-7F24-472E-9D49-1448562FD20E}" name="Resolved?" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{7DCAFC68-52C1-419F-AE79-351C1976AE51}" name="Resolution" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -494,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{239C0F2B-2F84-4D6A-8A50-2F86235AA26C}">
-  <dimension ref="A2:E30"/>
+  <dimension ref="A2:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.85546875" customWidth="1"/>
@@ -503,124 +594,198 @@
     <col min="5" max="5" width="51.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+    <row r="2" spans="1:5" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>2</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="4" spans="1:5" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:5" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
+    <row r="6" spans="1:5" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+    <row r="7" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
@@ -712,7 +877,16 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
     </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>